<commit_message>
docs: 1. Correct Spelling Mistake.
</commit_message>
<xml_diff>
--- a/Nutrients Template.xlsx
+++ b/Nutrients Template.xlsx
@@ -96,13 +96,7 @@
   </si>
   <si>
     <r>
-      <rPr>
-        <sz val="28"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <charset val="134"/>
-      </rPr>
-      <t>Systolic measurement has always been a main references of indicating whether a person has high blood presure or not. However by combining the Diastolic reading it is really hard to determine whether a person has high blood presure. According to the Medical associations Diastolic is the main causes of heart attack, heart stroke. Therefore the indications of the blood presure would be mainly base on </t>
+      <t>Systolic measurement has always been a main references of indicating whether a person has high blood pressure or not. However by combining the Diastolic reading it is really hard to determine whether a person has high blood pressure. According to the Medical associations Diastolic is the main causes of heart attack, heart stroke. Therefore the indications of the blood pressure would be mainly base on </t>
     </r>
     <r>
       <rPr>
@@ -185,7 +179,7 @@
     <t>Weight (lbs)</t>
   </si>
   <si>
-    <t>Blood Presure (mmHg)</t>
+    <t>Blood Pressure (mmHg)</t>
   </si>
   <si>
     <t>Oximeter</t>
@@ -924,16 +918,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="18"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial Regular"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <b/>
       <sz val="28"/>
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial Regular"/>
       <charset val="134"/>
     </font>
   </fonts>

</xml_diff>